<commit_message>
feat(vm-master): consolidate preview and sync workflow
</commit_message>
<xml_diff>
--- a/tests/fixtures/platform-api/groups_LTW_all.xlsx
+++ b/tests/fixtures/platform-api/groups_LTW_all.xlsx
@@ -13,7 +13,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
-    <t>群組</t>
+    <t>Group</t>
   </si>
   <si>
     <t>AD Account</t>
@@ -37,7 +37,7 @@
     <t>LEO.ZOU</t>
   </si>
   <si>
-    <t>鄒小明</t>
+    <t>Leo Zou</t>
   </si>
   <si>
     <t>leo.zou@deltaww.com</t>

</xml_diff>